<commit_message>
Update test case Excel files with steps on separate lines
- Modified Steps column to display each step on a separate line
- Increased row height to accommodate multi-line steps
- Improved readability for easier test execution
</commit_message>
<xml_diff>
--- a/Curation_Module_Test_Cases.xlsx
+++ b/Curation_Module_Test_Cases.xlsx
@@ -61,7 +61,11 @@
     <t>Maintenance and validation of column header mappings for Subject Summary files from different clinical studies</t>
   </si>
   <si>
-    <t>Step 1: User downloads the Column Header Mapping Excel file from the configuration folder. Step 2: User adds a new study protocol column (e.g. "GS-US-592-9999") with mappings for Subject, Site, Visit Date, Status, Last Visit. Step 3: User saves and uploads the updated mapping file to the configuration folder. Step 4: User uploads a Subject Summary file for study GS-US-592-9999 to the designated input folder for processing. Step 5: User verifies that curated output contains standardized column names (Subject, Site, Actual Visit Date, Subject Status, Last Visit).</t>
+    <t>Step 1: User downloads the Column Header Mapping Excel file from the configuration folder.
+Step 2: User adds a new study protocol column (e.g. "GS-US-592-9999") with mappings for Subject, Site, Visit Date, Status, Last Visit.
+Step 3: User saves and uploads the updated mapping file to the configuration folder.
+Step 4: User uploads a Subject Summary file for study GS-US-592-9999 to the designated input folder for processing.
+Step 5: User verifies that curated output contains standardized column names (Subject, Site, Actual Visit Date, Subject Status, Last Visit).</t>
   </si>
   <si>
     <t>Column Header Mapping Excel file (Header sheet)</t>
@@ -79,7 +83,12 @@
     <t>Processing a well-formatted Subject Summary file through the curation pipeline</t>
   </si>
   <si>
-    <t>Step 1: User places a Subject Summary CSV file in the designated date folder (e.g. 20251106) in the input location. Step 2: User initiates the curation process. Step 3: User navigates to the curated output location and opens the curated_subject_summary table. Step 4: User verifies that Study Protocol column is populated correctly (extracted from filename). Step 5: User verifies that column names match standardized names (Subject, Site, Actual Visit Date, Subject Status, etc.). Step 6: User verifies metadata columns are present: extract_date, processed_timestamp, source_file.</t>
+    <t>Step 1: User places a Subject Summary CSV file in the designated date folder (e.g. 20251106) in the input location.
+Step 2: User initiates the curation process.
+Step 3: User navigates to the curated output location and opens the curated_subject_summary table.
+Step 4: User verifies that Study Protocol column is populated correctly (extracted from filename).
+Step 5: User verifies that column names match standardized names (Subject, Site, Actual Visit Date, Subject Status, etc.).
+Step 6: User verifies metadata columns are present: extract_date, processed_timestamp, source_file.</t>
   </si>
   <si>
     <t>Subject Summary CSV file</t>
@@ -100,7 +109,11 @@
     <t>Validation that empty or sparse rows are removed during curation</t>
   </si>
   <si>
-    <t>Step 1: User prepares a Subject Summary file containing 5 rows with complete data and 3 rows with only 1-2 values populated. Step 2: User uploads the file to the input folder for processing. Step 3: User initiates the curation process. Step 4: User opens the curated output and counts the number of rows. Step 5: User verifies that only the 5 complete rows are present in the output, and sparse rows have been removed.</t>
+    <t>Step 1: User prepares a Subject Summary file containing 5 rows with complete data and 3 rows with only 1-2 values populated.
+Step 2: User uploads the file to the input folder for processing.
+Step 3: User initiates the curation process.
+Step 4: User opens the curated output and counts the number of rows.
+Step 5: User verifies that only the 5 complete rows are present in the output, and sparse rows have been removed.</t>
   </si>
   <si>
     <t>Subject Summary CSV file with sparse rows</t>
@@ -118,7 +131,11 @@
     <t>Validation that files with headers not on the first row are processed correctly</t>
   </si>
   <si>
-    <t>Step 1: User prepares a Subject Summary file where the actual header row is on row 5 (rows 1-4 contain export metadata or empty cells). Step 2: User uploads this file to the input folder. Step 3: User initiates the curation process. Step 4: User opens the curated output and verifies that data starts from the correct row. Step 5: User verifies that column mappings are applied correctly despite the offset header.</t>
+    <t>Step 1: User prepares a Subject Summary file where the actual header row is on row 5 (rows 1-4 contain export metadata or empty cells).
+Step 2: User uploads this file to the input folder.
+Step 3: User initiates the curation process.
+Step 4: User opens the curated output and verifies that data starts from the correct row.
+Step 5: User verifies that column mappings are applied correctly despite the offset header.</t>
   </si>
   <si>
     <t>Subject Summary CSV file with offset headers</t>
@@ -139,7 +156,11 @@
     <t>Validation that various date formats are converted to standardized output format</t>
   </si>
   <si>
-    <t>Step 1: User prepares a Subject Summary file with Visit Date column containing dates in different formats: "01-Jan-2025", "2025-01-01", "01 Jan 2025", "1/1/2025". Step 2: User uploads the file to the input folder. Step 3: User initiates the curation process. Step 4: User opens the curated output and examines the Actual Visit Date column. Step 5: User verifies all dates are converted to the standardized format (YYYY-MM-DD) regardless of input format.</t>
+    <t>Step 1: User prepares a Subject Summary file with Visit Date column containing dates in different formats: "01-Jan-2025", "2025-01-01", "01 Jan 2025", "1/1/2025".
+Step 2: User uploads the file to the input folder.
+Step 3: User initiates the curation process.
+Step 4: User opens the curated output and examines the Actual Visit Date column.
+Step 5: User verifies all dates are converted to the standardized format (YYYY-MM-DD) regardless of input format.</t>
   </si>
   <si>
     <t>Subject Summary CSV with mixed date formats</t>
@@ -160,7 +181,11 @@
     <t>Validation that extract_date metadata is correctly added to curated output</t>
   </si>
   <si>
-    <t>Step 1: User places a Subject Summary file in a dated folder named "20251106" in the input location. Step 2: User initiates the curation process. Step 3: User opens the curated output table. Step 4: User verifies that the extract_date column exists. Step 5: User verifies that all rows have extract_date value of "2025-11-06" matching the folder date.</t>
+    <t>Step 1: User places a Subject Summary file in a dated folder named "20251106" in the input location.
+Step 2: User initiates the curation process.
+Step 3: User opens the curated output table.
+Step 4: User verifies that the extract_date column exists.
+Step 5: User verifies that all rows have extract_date value of "2025-11-06" matching the folder date.</t>
   </si>
   <si>
     <t>File in folder 20251106</t>
@@ -175,7 +200,12 @@
     <t>Processing multiple Subject Summary files from different studies in a single batch</t>
   </si>
   <si>
-    <t>Step 1: User uploads 3 Subject Summary files from different studies (GS-US-592-6173, GS-US-380-5460, GS-US-123-4567) to the same input folder. Step 2: User initiates the curation process for batch processing. Step 3: User opens the curated output table. Step 4: User verifies that all 3 studies are present in the output (filters by Study Protocol column). Step 5: User verifies each study has correct column mappings applied based on the mapping file. Step 6: User verifies total row count matches combined input rows (minus sparse rows).</t>
+    <t>Step 1: User uploads 3 Subject Summary files from different studies (GS-US-592-6173, GS-US-380-5460, GS-US-123-4567) to the same input folder.
+Step 2: User initiates the curation process for batch processing.
+Step 3: User opens the curated output table.
+Step 4: User verifies that all 3 studies are present in the output (filters by Study Protocol column).
+Step 5: User verifies each study has correct column mappings applied based on the mapping file.
+Step 6: User verifies total row count matches combined input rows (minus sparse rows).</t>
   </si>
   <si>
     <t>Multiple Subject Summary CSV files</t>
@@ -193,7 +223,12 @@
     <t>Processing a Depot Inventory file through the curation pipeline</t>
   </si>
   <si>
-    <t>Step 1: User places a Depot Inventory CSV file in the designated date folder in the input location. Step 2: User initiates the curation process for depot inventory files. Step 3: User navigates to the curated output location and opens the curated_depot_inventory table. Step 4: User verifies that Study Protocol column is populated correctly. Step 5: User verifies that standard metadata columns are present (extract_date, processed_timestamp, source_file). Step 6: User verifies that depot-specific columns (Depot, Batch, Quantity Available, etc.) are preserved.</t>
+    <t>Step 1: User places a Depot Inventory CSV file in the designated date folder in the input location.
+Step 2: User initiates the curation process for depot inventory files.
+Step 3: User navigates to the curated output location and opens the curated_depot_inventory table.
+Step 4: User verifies that Study Protocol column is populated correctly.
+Step 5: User verifies that standard metadata columns are present (extract_date, processed_timestamp, source_file).
+Step 6: User verifies that depot-specific columns (Depot, Batch, Quantity Available, etc.) are preserved.</t>
   </si>
   <si>
     <t>Depot Inventory CSV file</t>
@@ -211,7 +246,12 @@
     <t>Processing a Site Inventory file through the curation pipeline</t>
   </si>
   <si>
-    <t>Step 1: User places a Site Inventory CSV file in the designated date folder in the input location. Step 2: User initiates the curation process for site inventory files. Step 3: User navigates to the curated output location and opens the curated_site_inventory table. Step 4: User verifies that Study Protocol column is populated correctly. Step 5: User verifies that standard metadata columns are present. Step 6: User verifies that site-specific columns (Site, Country, Batch, Quantity, etc.) are preserved.</t>
+    <t>Step 1: User places a Site Inventory CSV file in the designated date folder in the input location.
+Step 2: User initiates the curation process for site inventory files.
+Step 3: User navigates to the curated output location and opens the curated_site_inventory table.
+Step 4: User verifies that Study Protocol column is populated correctly.
+Step 5: User verifies that standard metadata columns are present.
+Step 6: User verifies that site-specific columns (Site, Country, Batch, Quantity, etc.) are preserved.</t>
   </si>
   <si>
     <t>Site Inventory CSV file</t>
@@ -229,7 +269,12 @@
     <t>Processing a Supply Method file through the curation pipeline</t>
   </si>
   <si>
-    <t>Step 1: User places a Supply Method CSV file in the designated date folder in the input location. Step 2: User initiates the curation process for supply method files. Step 3: User navigates to the curated output location and opens the curated_supply_method table. Step 4: User verifies that Study Protocol column is populated correctly. Step 5: User verifies that standard metadata columns are present. Step 6: User verifies that supply method data (Site/Country, Comparator Treatment, Supply Method) is preserved.</t>
+    <t>Step 1: User places a Supply Method CSV file in the designated date folder in the input location.
+Step 2: User initiates the curation process for supply method files.
+Step 3: User navigates to the curated output location and opens the curated_supply_method table.
+Step 4: User verifies that Study Protocol column is populated correctly.
+Step 5: User verifies that standard metadata columns are present.
+Step 6: User verifies that supply method data (Site/Country, Comparator Treatment, Supply Method) is preserved.</t>
   </si>
   <si>
     <t>Supply Method CSV file</t>
@@ -250,7 +295,11 @@
     <t>Validation of handling when a study protocol is not in the mapping file</t>
   </si>
   <si>
-    <t>Step 1: User uploads a Subject Summary file for a new study (GS-US-999-9999) that does not exist in the Column Header Mapping file. Step 2: User initiates the curation process. Step 3: User checks processing logs or error reports. Step 4: User verifies that system provides clear error message indicating missing mapping for study GS-US-999-9999. Step 5: User verifies that other studies in the same batch are still processed successfully.</t>
+    <t>Step 1: User uploads a Subject Summary file for a new study (GS-US-999-9999) that does not exist in the Column Header Mapping file.
+Step 2: User initiates the curation process.
+Step 3: User checks processing logs or error reports.
+Step 4: User verifies that system provides clear error message indicating missing mapping for study GS-US-999-9999.
+Step 5: User verifies that other studies in the same batch are still processed successfully.</t>
   </si>
   <si>
     <t>Subject Summary CSV for unmapped study</t>
@@ -268,7 +317,11 @@
     <t>Validation of handling when a required column is missing from input file</t>
   </si>
   <si>
-    <t>Step 1: User prepares a Subject Summary file missing the "Subject" column (critical required field). Step 2: User uploads the file to the input folder. Step 3: User initiates the curation process. Step 4: User checks processing logs or error reports. Step 5: User verifies that system provides clear error message indicating missing required column and which file is affected.</t>
+    <t>Step 1: User prepares a Subject Summary file missing the "Subject" column (critical required field).
+Step 2: User uploads the file to the input folder.
+Step 3: User initiates the curation process.
+Step 4: User checks processing logs or error reports.
+Step 5: User verifies that system provides clear error message indicating missing required column and which file is affected.</t>
   </si>
   <si>
     <t>Subject Summary CSV missing required column</t>
@@ -286,7 +339,11 @@
     <t>Validation of handling when a corrupted or non-CSV file is uploaded</t>
   </si>
   <si>
-    <t>Step 1: User accidentally uploads a corrupted file or wrong format file (e.g. .xlsx renamed to .csv, or file with binary content) to the input folder. Step 2: User initiates the curation process. Step 3: User checks processing logs or error reports. Step 4: User verifies that system provides clear error message indicating file format issue and which file is affected. Step 5: User verifies that other valid files in the same batch are still processed successfully.</t>
+    <t>Step 1: User accidentally uploads a corrupted file or wrong format file (e.g. .xlsx renamed to .csv, or file with binary content) to the input folder.
+Step 2: User initiates the curation process.
+Step 3: User checks processing logs or error reports.
+Step 4: User verifies that system provides clear error message indicating file format issue and which file is affected.
+Step 5: User verifies that other valid files in the same batch are still processed successfully.</t>
   </si>
   <si>
     <t>Corrupted CSV file</t>
@@ -307,7 +364,11 @@
     <t>Validation that all expected columns are present in curated output</t>
   </si>
   <si>
-    <t>Step 1: User reviews the expected standardized column list: Subject, Site, Actual Visit Date, Subject Status, Last Visit, Study Protocol, extract_date, processed_timestamp, source_file. Step 2: User processes a Subject Summary file through the curation pipeline. Step 3: User opens the curated output table. Step 4: User verifies that all expected standardized columns are present. Step 5: User verifies no unexpected columns are present (unless specified in mapping for additional passthrough columns).</t>
+    <t>Step 1: User reviews the expected standardized column list: Subject, Site, Actual Visit Date, Subject Status, Last Visit, Study Protocol, extract_date, processed_timestamp, source_file.
+Step 2: User processes a Subject Summary file through the curation pipeline.
+Step 3: User opens the curated output table.
+Step 4: User verifies that all expected standardized columns are present.
+Step 5: User verifies no unexpected columns are present (unless specified in mapping for additional passthrough columns).</t>
   </si>
   <si>
     <t>Standard GS-US-592-6173 file</t>
@@ -322,7 +383,12 @@
     <t>Validation that output row counts match input row counts (minus sparse rows)</t>
   </si>
   <si>
-    <t>Step 1: User prepares a Subject Summary file and manually counts total rows and sparse rows (rows with ≤2 values). Step 2: User calculates expected output row count = total rows - sparse rows. Step 3: User uploads the file and processes it through curation. Step 4: User opens the curated output and counts rows. Step 5: User verifies that output row count matches expected calculation. Step 6: User documents any discrepancies for investigation.</t>
+    <t>Step 1: User prepares a Subject Summary file and manually counts total rows and sparse rows (rows with ≤2 values).
+Step 2: User calculates expected output row count = total rows - sparse rows.
+Step 3: User uploads the file and processes it through curation.
+Step 4: User opens the curated output and counts rows.
+Step 5: User verifies that output row count matches expected calculation.
+Step 6: User documents any discrepancies for investigation.</t>
   </si>
   <si>
     <t>Subject Summary CSV with known row counts</t>
@@ -743,7 +809,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="100" customHeight="1">
+    <row r="2" spans="1:11" ht="150" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -770,7 +836,7 @@
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:11" ht="100" customHeight="1">
+    <row r="3" spans="1:11" ht="150" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -797,7 +863,7 @@
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
     </row>
-    <row r="4" spans="1:11" ht="100" customHeight="1">
+    <row r="4" spans="1:11" ht="150" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>24</v>
       </c>
@@ -824,7 +890,7 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:11" ht="100" customHeight="1">
+    <row r="5" spans="1:11" ht="150" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>31</v>
       </c>
@@ -851,7 +917,7 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:11" ht="100" customHeight="1">
+    <row r="6" spans="1:11" ht="150" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>37</v>
       </c>
@@ -878,7 +944,7 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
-    <row r="7" spans="1:11" ht="100" customHeight="1">
+    <row r="7" spans="1:11" ht="150" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>44</v>
       </c>
@@ -905,7 +971,7 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:11" ht="100" customHeight="1">
+    <row r="8" spans="1:11" ht="150" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>50</v>
       </c>
@@ -932,7 +998,7 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11" ht="100" customHeight="1">
+    <row r="9" spans="1:11" ht="150" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>56</v>
       </c>
@@ -959,7 +1025,7 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:11" ht="100" customHeight="1">
+    <row r="10" spans="1:11" ht="150" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>62</v>
       </c>
@@ -986,7 +1052,7 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:11" ht="100" customHeight="1">
+    <row r="11" spans="1:11" ht="150" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>68</v>
       </c>
@@ -1013,7 +1079,7 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:11" ht="100" customHeight="1">
+    <row r="12" spans="1:11" ht="150" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>74</v>
       </c>
@@ -1040,7 +1106,7 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:11" ht="100" customHeight="1">
+    <row r="13" spans="1:11" ht="150" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>81</v>
       </c>
@@ -1067,7 +1133,7 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="1:11" ht="100" customHeight="1">
+    <row r="14" spans="1:11" ht="150" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>87</v>
       </c>
@@ -1094,7 +1160,7 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:11" ht="100" customHeight="1">
+    <row r="15" spans="1:11" ht="150" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>93</v>
       </c>
@@ -1121,7 +1187,7 @@
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="1:11" ht="100" customHeight="1">
+    <row r="16" spans="1:11" ht="150" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>99</v>
       </c>

</xml_diff>